<commit_message>
Documentation: faculty mentor and status-mail dates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EGrnzrfHztmX7RAaosfXYG
</commit_message>
<xml_diff>
--- a/documentation/Nexus_Documentation/Nexus_Status_Report.xlsx
+++ b/documentation/Nexus_Documentation/Nexus_Status_Report.xlsx
@@ -879,7 +879,7 @@
       </c>
       <c r="D17" s="72" t="inlineStr">
         <is>
-          <t>[DD/MMM/YYYY]</t>
+          <t>27/Sep/2026</t>
         </is>
       </c>
     </row>
@@ -945,7 +945,7 @@
       </c>
       <c r="D23" s="72" t="inlineStr">
         <is>
-          <t>[DD/MMM/YYYY]</t>
+          <t>07/Oct/2026</t>
         </is>
       </c>
     </row>

</xml_diff>